<commit_message>
Add Task Category and fix category product
</commit_message>
<xml_diff>
--- a/testdata/CategoryProduct.xlsx
+++ b/testdata/CategoryProduct.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Sales Force\Automation\stp-automation-test\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A9C5BC5-4FA8-402A-9EE7-D895A64B85FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7A3C394-F5A6-42C1-BC65-63C18BBE97A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C7681F3F-D0BE-43DE-AC81-0EAE175E5E0E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C7681F3F-D0BE-43DE-AC81-0EAE175E5E0E}"/>
   </bookViews>
   <sheets>
     <sheet name="addCategoryProduct" sheetId="5" r:id="rId1"/>

</xml_diff>

<commit_message>
Add Customer and outlet
</commit_message>
<xml_diff>
--- a/testdata/CategoryProduct.xlsx
+++ b/testdata/CategoryProduct.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Sales Force\Automation\stp-automation-test\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7A3C394-F5A6-42C1-BC65-63C18BBE97A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C925E99E-EC97-4267-BD0C-BC9CEF585936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C7681F3F-D0BE-43DE-AC81-0EAE175E5E0E}"/>
   </bookViews>
@@ -46,13 +46,13 @@
     <t>CategoryName</t>
   </si>
   <si>
-    <t>Category 1</t>
+    <t>This category product was successfully changed</t>
   </si>
   <si>
-    <t>Category 2</t>
+    <t>Gadget</t>
   </si>
   <si>
-    <t>This category product was successfully changed</t>
+    <t>Cosmetic</t>
   </si>
 </sst>
 </file>
@@ -442,7 +442,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
@@ -482,10 +482,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
         <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -493,7 +493,7 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>